<commit_message>
data: first round lead search - 9 leads found (BGST, Thong Guan, logistics companies)
</commit_message>
<xml_diff>
--- a/sales-support/Sales_Hunter_Agent.xlsx
+++ b/sales-support/Sales_Hunter_Agent.xlsx
@@ -703,208 +703,622 @@
       <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
-      <c r="I5" s="5" t="n"/>
-      <c r="J5" s="5" t="n"/>
-      <c r="K5" s="5" t="n"/>
-      <c r="L5" s="5" t="n"/>
-      <c r="M5" s="5" t="n"/>
-      <c r="N5" s="5" t="n"/>
-      <c r="O5" s="6" t="n"/>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>BGST Resources Sdn Bhd</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Import/Export</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Small (11-50)</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>bgst.com.my</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr"/>
+      <c r="J5" s="5" t="inlineStr"/>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>Selangor, MY</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>Importer 进口商</t>
+        </is>
+      </c>
+      <c r="M5" s="5" t="inlineStr">
+        <is>
+          <t>Google Search</t>
+        </is>
+      </c>
+      <c r="N5" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="O5" s="6" t="inlineStr">
+        <is>
+          <t>New 新</t>
+        </is>
+      </c>
       <c r="P5" s="6" t="n"/>
       <c r="Q5" s="6" t="n"/>
       <c r="R5" s="5" t="n"/>
-      <c r="S5" s="5" t="n"/>
+      <c r="S5" s="5" t="inlineStr">
+        <is>
+          <t>马来西亚进口公司，专做中国采购+海运，10年+经验，2500+学员，注册海关代理+MATRADE认证。直接竞争对手？或合作伙伴机会。</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
-      <c r="I6" s="5" t="n"/>
-      <c r="J6" s="5" t="n"/>
-      <c r="K6" s="5" t="n"/>
-      <c r="L6" s="5" t="n"/>
-      <c r="M6" s="5" t="n"/>
-      <c r="N6" s="5" t="n"/>
-      <c r="O6" s="6" t="n"/>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Thong Guan Industries Berhad</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Manufacturing/Packaging</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Medium (51-250)</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>thongguan.com</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr"/>
+      <c r="J6" s="5" t="inlineStr"/>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>Penang, MY</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>Exporter 出口商</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>Google Search</t>
+        </is>
+      </c>
+      <c r="N6" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="O6" s="6" t="inlineStr">
+        <is>
+          <t>New 新</t>
+        </is>
+      </c>
       <c r="P6" s="6" t="n"/>
       <c r="Q6" s="6" t="n"/>
       <c r="R6" s="5" t="n"/>
-      <c r="S6" s="5" t="n"/>
+      <c r="S6" s="5" t="inlineStr">
+        <is>
+          <t>马来西亚最大拉伸膜制造商，1942年成立，出口到60+国家。需要稳定的出口海运服务。</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
-      <c r="I7" s="5" t="n"/>
-      <c r="J7" s="5" t="n"/>
-      <c r="K7" s="5" t="n"/>
-      <c r="L7" s="5" t="n"/>
-      <c r="M7" s="5" t="n"/>
-      <c r="N7" s="5" t="n"/>
-      <c r="O7" s="6" t="n"/>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>JUST SHIP Logistics Sdn Bhd</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Logistics/Freight</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Small (11-50)</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>yellowpages.my</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr"/>
+      <c r="J7" s="5" t="inlineStr"/>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>Kuching, Sarawak</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>Both 进出口</t>
+        </is>
+      </c>
+      <c r="M7" s="5" t="inlineStr">
+        <is>
+          <t>Yellow Pages</t>
+        </is>
+      </c>
+      <c r="N7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="O7" s="6" t="inlineStr">
+        <is>
+          <t>New 新</t>
+        </is>
+      </c>
       <c r="P7" s="6" t="n"/>
       <c r="Q7" s="6" t="n"/>
       <c r="R7" s="5" t="n"/>
-      <c r="S7" s="5" t="n"/>
+      <c r="S7" s="5" t="inlineStr">
+        <is>
+          <t>货运代理公司，古晋。可能是同行合作伙伴或需要东南亚转运支持。</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
-      <c r="I8" s="5" t="n"/>
-      <c r="J8" s="5" t="n"/>
-      <c r="K8" s="5" t="n"/>
-      <c r="L8" s="5" t="n"/>
-      <c r="M8" s="5" t="n"/>
-      <c r="N8" s="5" t="n"/>
-      <c r="O8" s="6" t="n"/>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>SWCOM Logistics Sdn Bhd</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Logistics/Freight</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Small (11-50)</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>yellowpages.my</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr"/>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr"/>
+      <c r="J8" s="5" t="inlineStr"/>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Labuan, MY</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Both 进出口</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Yellow Pages</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="O8" s="6" t="inlineStr">
+        <is>
+          <t>New 新</t>
+        </is>
+      </c>
       <c r="P8" s="6" t="n"/>
       <c r="Q8" s="6" t="n"/>
       <c r="R8" s="5" t="n"/>
-      <c r="S8" s="5" t="n"/>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>100% Bumiputera 公司，清关+仓储+运输+船务代理。纳闽自贸区。</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
-      <c r="I9" s="5" t="n"/>
-      <c r="J9" s="5" t="n"/>
-      <c r="K9" s="5" t="n"/>
-      <c r="L9" s="5" t="n"/>
-      <c r="M9" s="5" t="n"/>
-      <c r="N9" s="5" t="n"/>
-      <c r="O9" s="6" t="n"/>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Hyper Shipping Sdn Bhd</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Logistics/Freight</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Small (11-50)</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>yellowpages.my</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr"/>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr"/>
+      <c r="J9" s="5" t="inlineStr"/>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>Bintulu, Sarawak</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>Both 进出口</t>
+        </is>
+      </c>
+      <c r="M9" s="5" t="inlineStr">
+        <is>
+          <t>Yellow Pages</t>
+        </is>
+      </c>
+      <c r="N9" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="O9" s="6" t="inlineStr">
+        <is>
+          <t>New 新</t>
+        </is>
+      </c>
       <c r="P9" s="6" t="n"/>
       <c r="Q9" s="6" t="n"/>
       <c r="R9" s="5" t="n"/>
-      <c r="S9" s="5" t="n"/>
+      <c r="S9" s="5" t="inlineStr">
+        <is>
+          <t>货运代理，民都鲁，18年经验，主做砂拉越市场。</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
-      <c r="I10" s="5" t="n"/>
-      <c r="J10" s="5" t="n"/>
-      <c r="K10" s="5" t="n"/>
-      <c r="L10" s="5" t="n"/>
-      <c r="M10" s="5" t="n"/>
-      <c r="N10" s="5" t="n"/>
-      <c r="O10" s="6" t="n"/>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Capricorn Freight Services Sdn Bhd</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Logistics/Freight</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Small (11-50)</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>yellowpages.my</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr"/>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr"/>
+      <c r="J10" s="5" t="inlineStr"/>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>Kota Kinabalu, Sabah</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>Both 进出口</t>
+        </is>
+      </c>
+      <c r="M10" s="5" t="inlineStr">
+        <is>
+          <t>Yellow Pages</t>
+        </is>
+      </c>
+      <c r="N10" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="O10" s="6" t="inlineStr">
+        <is>
+          <t>New 新</t>
+        </is>
+      </c>
       <c r="P10" s="6" t="n"/>
       <c r="Q10" s="6" t="n"/>
       <c r="R10" s="5" t="n"/>
-      <c r="S10" s="5" t="n"/>
+      <c r="S10" s="5" t="inlineStr">
+        <is>
+          <t>货运代理，亚庇，沙巴市场。</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n"/>
-      <c r="I11" s="5" t="n"/>
-      <c r="J11" s="5" t="n"/>
-      <c r="K11" s="5" t="n"/>
-      <c r="L11" s="5" t="n"/>
-      <c r="M11" s="5" t="n"/>
-      <c r="N11" s="5" t="n"/>
-      <c r="O11" s="6" t="n"/>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Soon Tat Transport Sdn Bhd</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Logistics/Transport</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Small (11-50)</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>yellowpages.my</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr"/>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr"/>
+      <c r="J11" s="5" t="inlineStr"/>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>Puchong, Selangor</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>Both 进出口</t>
+        </is>
+      </c>
+      <c r="M11" s="5" t="inlineStr">
+        <is>
+          <t>Yellow Pages</t>
+        </is>
+      </c>
+      <c r="N11" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="O11" s="6" t="inlineStr">
+        <is>
+          <t>New 新</t>
+        </is>
+      </c>
       <c r="P11" s="6" t="n"/>
       <c r="Q11" s="6" t="n"/>
       <c r="R11" s="5" t="n"/>
-      <c r="S11" s="5" t="n"/>
+      <c r="S11" s="5" t="inlineStr">
+        <is>
+          <t>运输公司，蒲种，雪兰莪。</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="5" t="n"/>
-      <c r="H12" s="5" t="n"/>
-      <c r="I12" s="5" t="n"/>
-      <c r="J12" s="5" t="n"/>
-      <c r="K12" s="5" t="n"/>
-      <c r="L12" s="5" t="n"/>
-      <c r="M12" s="5" t="n"/>
-      <c r="N12" s="5" t="n"/>
-      <c r="O12" s="6" t="n"/>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>SVI Global</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Sourcing/Trading</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Small (11-50)</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>svigloballtd.com</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr"/>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr"/>
+      <c r="J12" s="5" t="inlineStr"/>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>Malaysia</t>
+        </is>
+      </c>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>Both 进出口</t>
+        </is>
+      </c>
+      <c r="M12" s="5" t="inlineStr">
+        <is>
+          <t>Google Search</t>
+        </is>
+      </c>
+      <c r="N12" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="O12" s="6" t="inlineStr">
+        <is>
+          <t>New 新</t>
+        </is>
+      </c>
       <c r="P12" s="6" t="n"/>
       <c r="Q12" s="6" t="n"/>
       <c r="R12" s="5" t="n"/>
-      <c r="S12" s="5" t="n"/>
+      <c r="S12" s="5" t="inlineStr">
+        <is>
+          <t>马来西亚采购代理，帮企业找中国供应商，做sourcing几十年。</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="5" t="n"/>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="5" t="n"/>
-      <c r="I13" s="5" t="n"/>
-      <c r="J13" s="5" t="n"/>
-      <c r="K13" s="5" t="n"/>
-      <c r="L13" s="5" t="n"/>
-      <c r="M13" s="5" t="n"/>
-      <c r="N13" s="5" t="n"/>
-      <c r="O13" s="6" t="n"/>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>CNMY Logistics</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Logistics/Freight</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Small (11-50)</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>cnmylogistics.com</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr"/>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr"/>
+      <c r="J13" s="5" t="inlineStr"/>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>Malaysia</t>
+        </is>
+      </c>
+      <c r="L13" s="5" t="inlineStr">
+        <is>
+          <t>Both 进出口</t>
+        </is>
+      </c>
+      <c r="M13" s="5" t="inlineStr">
+        <is>
+          <t>Google Search</t>
+        </is>
+      </c>
+      <c r="N13" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="O13" s="6" t="inlineStr">
+        <is>
+          <t>New 新</t>
+        </is>
+      </c>
       <c r="P13" s="6" t="n"/>
       <c r="Q13" s="6" t="n"/>
       <c r="R13" s="5" t="n"/>
-      <c r="S13" s="5" t="n"/>
+      <c r="S13" s="5" t="inlineStr">
+        <is>
+          <t>中马专线空运/海运，服务电商卖家和采购代理。</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">

</xml_diff>